<commit_message>
feat(divergent-universe): author source decks and compile card instances
Preserve nine explicit source-deck selections, 125 distinct instances and 15 preset joins through openpyxl, Sora and typed catalogs. Compile selected decks through the production factory without claiming mask eligibility or complete route integration.

Verify data rejection cases, shared-activity deck execution, fresh reconstruction and Sora drift. Refresh current public replay seeds for the changed decision identity.
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -34,13 +34,15 @@
     <sheet name="CurioDomainGrants" sheetId="25" r:id="rId25"/>
     <sheet name="EquationExpansionRewards" sheetId="26" r:id="rId26"/>
     <sheet name="DomainLayout" sheetId="27" r:id="rId27"/>
+    <sheet name="DomainDecks" sheetId="28" r:id="rId28"/>
+    <sheet name="DomainCards" sheetId="29" r:id="rId29"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1946" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2065" uniqueCount="224">
   <si>
     <t>@table</t>
   </si>
@@ -676,6 +678,42 @@
   </si>
   <si>
     <t>enum&lt;DuDomainSlotKind&gt;</t>
+  </si>
+  <si>
+    <t>DuDomainDecks</t>
+  </si>
+  <si>
+    <t>dffd7b16ec599e1f</t>
+  </si>
+  <si>
+    <t>style_source</t>
+  </si>
+  <si>
+    <t>card_count</t>
+  </si>
+  <si>
+    <t>enum&lt;DuDomainDeckPolicy&gt;</t>
+  </si>
+  <si>
+    <t>range=1..256</t>
+  </si>
+  <si>
+    <t>DuDomainCards</t>
+  </si>
+  <si>
+    <t>5022e055fa084725</t>
+  </si>
+  <si>
+    <t>deck_id</t>
+  </si>
+  <si>
+    <t>ref&lt;DuDomainDecks.id&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuDomainCardKind&gt;</t>
+  </si>
+  <si>
+    <t>range=1..5</t>
   </si>
 </sst>
 </file>
@@ -6856,6 +6894,482 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="12.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExplicitSourceDeck" promptTitle="DuDomainDeckPolicy enum" prompt="Select a value from the dropdown." sqref="E8:E1007">
+      <formula1>"ExplicitSourceDeck"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 256." promptTitle="Integer range" prompt="Enter an integer from 1 to 256." sqref="F8:F1007">
+      <formula1>1</formula1>
+      <formula2>256</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 256." promptTitle="Integer range" prompt="Enter an integer from 1 to 256." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>256</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Battle, Encounter, Event, Coin, Shop, Reward, Adventure, Reforge, Elite" promptTitle="DuDomainCardKind enum" prompt="Select a value from the dropdown." sqref="G8:G1007">
+      <formula1>"Battle,Encounter,Event,Coin,Shop,Reward,Adventure,Reforge,Elite"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 5." promptTitle="Integer range" prompt="Enter an integer from 1 to 5." sqref="H8:H1007">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): load authored shop stock from production sora
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -36,13 +36,15 @@
     <sheet name="DomainLayout" sheetId="27" r:id="rId27"/>
     <sheet name="DomainDecks" sheetId="28" r:id="rId28"/>
     <sheet name="DomainCards" sheetId="29" r:id="rId29"/>
+    <sheet name="ShopStocks" sheetId="30" r:id="rId30"/>
+    <sheet name="ShopItems" sheetId="31" r:id="rId31"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2065" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2169" uniqueCount="235">
   <si>
     <t>@table</t>
   </si>
@@ -714,6 +716,39 @@
   </si>
   <si>
     <t>range=1..5</t>
+  </si>
+  <si>
+    <t>DuShopStocks</t>
+  </si>
+  <si>
+    <t>15003b1e2dd908c4</t>
+  </si>
+  <si>
+    <t>enum&lt;DuShopStockPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuShopItems</t>
+  </si>
+  <si>
+    <t>32462bf5e4f1062f</t>
+  </si>
+  <si>
+    <t>stock_id</t>
+  </si>
+  <si>
+    <t>reward_kind</t>
+  </si>
+  <si>
+    <t>reward_key</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>ref&lt;DuShopStocks.id&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuShopRewardKind&gt;</t>
   </si>
 </sst>
 </file>
@@ -7550,6 +7585,424 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExplicitFixedStockAndPriceBaseRewards" promptTitle="DuShopStockPolicy enum" prompt="Select a value from the dropdown." sqref="D8:D1007">
+      <formula1>"ExplicitFixedStockAndPriceBaseRewards"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="5" customWidth="1"/>
+    <col min="7" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Blessing, Curio" promptTitle="DuShopRewardKind enum" prompt="Select a value from the dropdown." sqref="F8:F1007">
+      <formula1>"Blessing,Curio"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute authored wealth chest pickups
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -38,13 +38,14 @@
     <sheet name="DomainCards" sheetId="29" r:id="rId29"/>
     <sheet name="ShopStocks" sheetId="30" r:id="rId30"/>
     <sheet name="ShopItems" sheetId="31" r:id="rId31"/>
+    <sheet name="CoinRewards" sheetId="32" r:id="rId32"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2169" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2239" uniqueCount="238">
   <si>
     <t>@table</t>
   </si>
@@ -749,6 +750,15 @@
   </si>
   <si>
     <t>enum&lt;DuShopRewardKind&gt;</t>
+  </si>
+  <si>
+    <t>DuCoinRewards</t>
+  </si>
+  <si>
+    <t>c4bf737b5b73e514</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCoinRewardPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -8003,6 +8013,277 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="5" customWidth="1"/>
+    <col min="5" max="6" width="12.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="24.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 5." promptTitle="Integer range" prompt="Enter an integer from 1 to 5." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: FixedSingleChestCreditNoAmusementFacilities" promptTitle="DuCoinRewardPolicy enum" prompt="Select a value from the dropdown." sqref="G8:G1007">
+      <formula1>"FixedSingleChestCreditNoAmusementFacilities"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute authored reward-card occurrences
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -39,13 +39,14 @@
     <sheet name="ShopStocks" sheetId="30" r:id="rId30"/>
     <sheet name="ShopItems" sheetId="31" r:id="rId31"/>
     <sheet name="CoinRewards" sheetId="32" r:id="rId32"/>
+    <sheet name="RewardOccurrences" sheetId="33" r:id="rId33"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2239" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2308" uniqueCount="241">
   <si>
     <t>@table</t>
   </si>
@@ -759,6 +760,15 @@
   </si>
   <si>
     <t>enum&lt;DuCoinRewardPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuRewardOccurrences</t>
+  </si>
+  <si>
+    <t>0545eb170f7529e1</t>
+  </si>
+  <si>
+    <t>enum&lt;DuRewardOccurrencePolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -8284,6 +8294,276 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="29.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 5." promptTitle="Integer range" prompt="Enter an integer from 1 to 5." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: SingleExplicitRewardOnlySubstituteNoPoolSampling" promptTitle="DuRewardOccurrencePolicy enum" prompt="Select a value from the dropdown." sqref="G8:G1007">
+      <formula1>"SingleExplicitRewardOnlySubstituteNoPoolSampling"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): settle authored adventure chest results
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -40,13 +40,14 @@
     <sheet name="ShopItems" sheetId="31" r:id="rId31"/>
     <sheet name="CoinRewards" sheetId="32" r:id="rId32"/>
     <sheet name="RewardOccurrences" sheetId="33" r:id="rId33"/>
+    <sheet name="AdventureRewards" sheetId="34" r:id="rId34"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2308" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2383" uniqueCount="246">
   <si>
     <t>@table</t>
   </si>
@@ -769,6 +770,21 @@
   </si>
   <si>
     <t>enum&lt;DuRewardOccurrencePolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuAdventureRewards</t>
+  </si>
+  <si>
+    <t>6056789b0fbbcef6</t>
+  </si>
+  <si>
+    <t>maximum_chests</t>
+  </si>
+  <si>
+    <t>fragments_per_chest</t>
+  </si>
+  <si>
+    <t>enum&lt;DuAdventureRewardPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -8564,6 +8580,299 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="29.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 5." promptTitle="Integer range" prompt="Enter an integer from 1 to 5." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 3." promptTitle="Integer range" prompt="Enter an integer from 1 to 3." sqref="F8:F1007">
+      <formula1>1</formula1>
+      <formula2>3</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExternalEarnedChestCountAggregateFragmentsOnly" promptTitle="DuAdventureRewardPolicy enum" prompt="Select a value from the dropdown." sqref="H8:H1007">
+      <formula1>"ExternalEarnedChestCountAggregateFragmentsOnly"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute weighted curio hunt splash
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -41,13 +41,14 @@
     <sheet name="CoinRewards" sheetId="32" r:id="rId32"/>
     <sheet name="RewardOccurrences" sheetId="33" r:id="rId33"/>
     <sheet name="AdventureRewards" sheetId="34" r:id="rId34"/>
+    <sheet name="WeightedCurioSplashes" sheetId="35" r:id="rId35"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2383" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2463" uniqueCount="254">
   <si>
     <t>@table</t>
   </si>
@@ -785,6 +786,30 @@
   </si>
   <si>
     <t>enum&lt;DuAdventureRewardPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioSplashes</t>
+  </si>
+  <si>
+    <t>e8562d10ab8b36e1</t>
+  </si>
+  <si>
+    <t>weighted_curio_key</t>
+  </si>
+  <si>
+    <t>maze_buff_id</t>
+  </si>
+  <si>
+    <t>character_path</t>
+  </si>
+  <si>
+    <t>fraction_parameter</t>
+  </si>
+  <si>
+    <t>damage_fraction</t>
+  </si>
+  <si>
+    <t>enum&lt;DuWeightedCurioSplashPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -8873,6 +8898,312 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="32.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: HitCalculatedCopyAdjacentTrueDamage" promptTitle="DuWeightedCurioSplashPolicy enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
+      <formula1>"HitCalculatedCopyAdjacentTrueDamage"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute harmony weighted curio shields
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -42,13 +42,14 @@
     <sheet name="RewardOccurrences" sheetId="33" r:id="rId33"/>
     <sheet name="AdventureRewards" sheetId="34" r:id="rId34"/>
     <sheet name="WeightedCurioSplashes" sheetId="35" r:id="rId35"/>
+    <sheet name="WeightedCurioShields" sheetId="36" r:id="rId36"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2463" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2553" uniqueCount="260">
   <si>
     <t>@table</t>
   </si>
@@ -810,6 +811,24 @@
   </si>
   <si>
     <t>enum&lt;DuWeightedCurioSplashPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioShields</t>
+  </si>
+  <si>
+    <t>ff5977a6e4b4c06f</t>
+  </si>
+  <si>
+    <t>shield_fraction</t>
+  </si>
+  <si>
+    <t>duration_parameter</t>
+  </si>
+  <si>
+    <t>duration_turns</t>
+  </si>
+  <si>
+    <t>enum&lt;DuWeightedCurioShieldPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -9204,6 +9223,354 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="32.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="21.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="J8:J1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AllyActionResolvedReplaceTargetTurnShield" promptTitle="DuWeightedCurioShieldPolicy enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AllyActionResolvedReplaceTargetTurnShield"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute the story presently bonuses
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -44,13 +44,14 @@
     <sheet name="WeightedCurioSplashes" sheetId="35" r:id="rId35"/>
     <sheet name="WeightedCurioShields" sheetId="36" r:id="rId36"/>
     <sheet name="WeightedCurioAttackDebuffs" sheetId="37" r:id="rId37"/>
+    <sheet name="WeightedCurioSupportAttacks" sheetId="38" r:id="rId38"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2653" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2753" uniqueCount="277">
   <si>
     <t>@table</t>
   </si>
@@ -854,6 +855,33 @@
   </si>
   <si>
     <t>enum&lt;DuCurioAttackDebuffPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioSupportAttacks</t>
+  </si>
+  <si>
+    <t>8c8d15811d86d472</t>
+  </si>
+  <si>
+    <t>crit_rate_parameter</t>
+  </si>
+  <si>
+    <t>crit_rate_fraction</t>
+  </si>
+  <si>
+    <t>crit_damage_parameter</t>
+  </si>
+  <si>
+    <t>crit_damage_fraction</t>
+  </si>
+  <si>
+    <t>additional_parameter</t>
+  </si>
+  <si>
+    <t>additional_multiplier</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioSupportAttackPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -9981,6 +10009,387 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" style="5" customWidth="1"/>
+    <col min="10" max="11" width="20.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="32.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: RosterCountCritAndAttackResolvedAdditional" promptTitle="DuCurioSupportAttackPolicy enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"RosterCountCritAndAttackResolvedAdditional"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute road of prayers resource effects
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -45,13 +45,14 @@
     <sheet name="WeightedCurioShields" sheetId="36" r:id="rId36"/>
     <sheet name="WeightedCurioAttackDebuffs" sheetId="37" r:id="rId37"/>
     <sheet name="WeightedCurioSupportAttacks" sheetId="38" r:id="rId38"/>
+    <sheet name="WeightedCurioPrayers" sheetId="39" r:id="rId39"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2753" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="285">
   <si>
     <t>@table</t>
   </si>
@@ -882,6 +883,30 @@
   </si>
   <si>
     <t>enum&lt;DuCurioSupportAttackPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioPrayers</t>
+  </si>
+  <si>
+    <t>167c53616f8ef2cd</t>
+  </si>
+  <si>
+    <t>hp_parameter</t>
+  </si>
+  <si>
+    <t>hp_fraction</t>
+  </si>
+  <si>
+    <t>consume_parameter</t>
+  </si>
+  <si>
+    <t>consume_fraction</t>
+  </si>
+  <si>
+    <t>shield_parameter</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioPrayerPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -10390,6 +10415,386 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" style="5" customWidth="1"/>
+    <col min="10" max="11" width="16.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: EntryHpAndTurnStartConsumeShield" promptTitle="DuCurioPrayerPolicy enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"EntryHpAndTurnStartConsumeShield"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute self-amusement retaliation
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -46,13 +46,14 @@
     <sheet name="WeightedCurioAttackDebuffs" sheetId="37" r:id="rId37"/>
     <sheet name="WeightedCurioSupportAttacks" sheetId="38" r:id="rId38"/>
     <sheet name="WeightedCurioPrayers" sheetId="39" r:id="rId39"/>
+    <sheet name="WeightedCurioRetaliations" sheetId="40" r:id="rId40"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="300">
   <si>
     <t>@table</t>
   </si>
@@ -907,6 +908,51 @@
   </si>
   <si>
     <t>enum&lt;DuCurioPrayerPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioRetaliations</t>
+  </si>
+  <si>
+    <t>55e830dc5f843182</t>
+  </si>
+  <si>
+    <t>character_elements</t>
+  </si>
+  <si>
+    <t>aggro_parameter</t>
+  </si>
+  <si>
+    <t>aggro_fraction</t>
+  </si>
+  <si>
+    <t>base_aggro_destruction</t>
+  </si>
+  <si>
+    <t>base_aggro_hunt</t>
+  </si>
+  <si>
+    <t>base_aggro_erudition</t>
+  </si>
+  <si>
+    <t>base_aggro_harmony</t>
+  </si>
+  <si>
+    <t>base_aggro_nihility</t>
+  </si>
+  <si>
+    <t>base_aggro_preservation</t>
+  </si>
+  <si>
+    <t>base_aggro_abundance</t>
+  </si>
+  <si>
+    <t>base_aggro_remembrance</t>
+  </si>
+  <si>
+    <t>base_aggro_elation</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioRetaliationPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -11013,6 +11059,503 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Y7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="18.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="23.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="22.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="30.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="12.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="13.7109375" style="5" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" style="5" customWidth="1"/>
+    <col min="24" max="24" width="21.7109375" style="5" customWidth="1"/>
+    <col min="25" max="25" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: PhysicalAggroAndOwnerAdditional" promptTitle="DuCurioRetaliationPolicy enum" prompt="Select a value from the dropdown." sqref="T8:T1007">
+      <formula1>"PhysicalAggroAndOwnerAdditional"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute converse of entropy
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -47,13 +47,14 @@
     <sheet name="WeightedCurioSupportAttacks" sheetId="38" r:id="rId38"/>
     <sheet name="WeightedCurioPrayers" sheetId="39" r:id="rId39"/>
     <sheet name="WeightedCurioRetaliations" sheetId="40" r:id="rId40"/>
+    <sheet name="WeightedCurioBreakEffects" sheetId="41" r:id="rId41"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3068" uniqueCount="305">
   <si>
     <t>@table</t>
   </si>
@@ -953,6 +954,21 @@
   </si>
   <si>
     <t>enum&lt;DuCurioRetaliationPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioBreakEffects</t>
+  </si>
+  <si>
+    <t>0f1880a1a9067e77</t>
+  </si>
+  <si>
+    <t>multiplier_parameter</t>
+  </si>
+  <si>
+    <t>multiplier</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioBreakEffectPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -11556,6 +11572,312 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: EntryHighestTeamBreakEffectCapture" promptTitle="DuCurioBreakEffectPolicy enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
+      <formula1>"EntryHighestTeamBreakEffectCapture"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): execute mock crimson moon
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -48,13 +48,14 @@
     <sheet name="WeightedCurioPrayers" sheetId="39" r:id="rId39"/>
     <sheet name="WeightedCurioRetaliations" sheetId="40" r:id="rId40"/>
     <sheet name="WeightedCurioBreakEffects" sheetId="41" r:id="rId41"/>
+    <sheet name="WeightedCurioNecroses" sheetId="42" r:id="rId42"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3068" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3178" uniqueCount="314">
   <si>
     <t>@table</t>
   </si>
@@ -969,6 +970,33 @@
   </si>
   <si>
     <t>enum&lt;DuCurioBreakEffectPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioNecroses</t>
+  </si>
+  <si>
+    <t>c3af3f1bfed9abb2</t>
+  </si>
+  <si>
+    <t>chance_parameter</t>
+  </si>
+  <si>
+    <t>base_chance</t>
+  </si>
+  <si>
+    <t>damage_parameter</t>
+  </si>
+  <si>
+    <t>attack_multiplier</t>
+  </si>
+  <si>
+    <t>detonation_parameter</t>
+  </si>
+  <si>
+    <t>detonation_fraction</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioNecrosisPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -11878,6 +11906,430 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="27.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="21.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="7">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="L8:L1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="M8:M1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AttackResolvedNecrosisAndDotDamageBurnDetonation" promptTitle="DuCurioNecrosisPolicy enum" prompt="Select a value from the dropdown." sqref="O8:O1007">
+      <formula1>"AttackResolvedNecrosisAndDotDamageBurnDetonation"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): g22-p5-b2 author sapient pen operands
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -49,13 +49,14 @@
     <sheet name="WeightedCurioRetaliations" sheetId="40" r:id="rId40"/>
     <sheet name="WeightedCurioBreakEffects" sheetId="41" r:id="rId41"/>
     <sheet name="WeightedCurioNecroses" sheetId="42" r:id="rId42"/>
+    <sheet name="WeightedCurioElations" sheetId="43" r:id="rId43"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3178" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3278" uniqueCount="320">
   <si>
     <t>@table</t>
   </si>
@@ -997,6 +998,24 @@
   </si>
   <si>
     <t>enum&lt;DuCurioNecrosisPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioElations</t>
+  </si>
+  <si>
+    <t>63b66e242e9964f7</t>
+  </si>
+  <si>
+    <t>gain_parameter</t>
+  </si>
+  <si>
+    <t>punchline_gain</t>
+  </si>
+  <si>
+    <t>elation_bonus</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioElationPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -12330,6 +12349,395 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="8" width="14.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="26.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="7">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="H8:H1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="L8:L1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ActionResolvedOriginalPartyRefresh" promptTitle="DuCurioElationPolicy enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"ActionResolvedOriginalPartyRefresh"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): g22-p5-b2 assemble shared punchline resource
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -50,13 +50,14 @@
     <sheet name="WeightedCurioBreakEffects" sheetId="41" r:id="rId41"/>
     <sheet name="WeightedCurioNecroses" sheetId="42" r:id="rId42"/>
     <sheet name="WeightedCurioElations" sheetId="43" r:id="rId43"/>
+    <sheet name="BattleTeamResources" sheetId="44" r:id="rId44"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3278" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3353" uniqueCount="327">
   <si>
     <t>@table</t>
   </si>
@@ -1016,6 +1017,27 @@
   </si>
   <si>
     <t>enum&lt;DuCurioElationPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuBattleTeamResources</t>
+  </si>
+  <si>
+    <t>0ccaeb7a31908794</t>
+  </si>
+  <si>
+    <t>resource_key</t>
+  </si>
+  <si>
+    <t>initial_value</t>
+  </si>
+  <si>
+    <t>maximum_value</t>
+  </si>
+  <si>
+    <t>enum&lt;DuBattleTeamResourcePolicy&gt;</t>
+  </si>
+  <si>
+    <t>range=0..65535</t>
   </si>
 </sst>
 </file>
@@ -12738,6 +12760,297 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="12.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="13.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 65535." promptTitle="Integer range" prompt="Enter an integer from 0 to 65535." sqref="F8:F1007">
+      <formula1>0</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: OriginalElationZeroClampPersist" promptTitle="DuBattleTeamResourcePolicy enum" prompt="Select a value from the dropdown." sqref="H8:H1007">
+      <formula1>"OriginalElationZeroClampPersist"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(divergent-universe): g22-p5-b2 author genius confusion operands
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -51,13 +51,14 @@
     <sheet name="WeightedCurioNecroses" sheetId="42" r:id="rId42"/>
     <sheet name="WeightedCurioElations" sheetId="43" r:id="rId43"/>
     <sheet name="BattleTeamResources" sheetId="44" r:id="rId44"/>
+    <sheet name="WeightedCurioExcitations" sheetId="45" r:id="rId45"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3353" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3478" uniqueCount="333">
   <si>
     <t>@table</t>
   </si>
@@ -1038,6 +1039,24 @@
   </si>
   <si>
     <t>range=0..65535</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioExcitations</t>
+  </si>
+  <si>
+    <t>72b8aabd7498ebac</t>
+  </si>
+  <si>
+    <t>stack_gain</t>
+  </si>
+  <si>
+    <t>stack_consumption</t>
+  </si>
+  <si>
+    <t>policy_maximum_stacks</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioExcitationPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -13051,6 +13070,496 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:W7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="5" customWidth="1"/>
+    <col min="9" max="10" width="17.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="18.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="29.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="12.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="13.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="12.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="21.7109375" style="5" customWidth="1"/>
+    <col min="23" max="23" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="11">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="H8:H1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="J8:J1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="M8:M1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="O8:O1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="P8:P1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="Q8:Q1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: EffectiveGainActionResolvedTeamConsumption" promptTitle="DuCurioExcitationPolicy enum" prompt="Select a value from the dropdown." sqref="R8:R1007">
+      <formula1>"EffectiveGainActionResolvedTeamConsumption"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(universe): author weighted curio encouragement operands
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -52,13 +52,14 @@
     <sheet name="WeightedCurioElations" sheetId="43" r:id="rId43"/>
     <sheet name="BattleTeamResources" sheetId="44" r:id="rId44"/>
     <sheet name="WeightedCurioExcitations" sheetId="45" r:id="rId45"/>
+    <sheet name="WeightedCurioEncouragements" sheetId="46" r:id="rId46"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3478" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3558" uniqueCount="338">
   <si>
     <t>@table</t>
   </si>
@@ -1057,6 +1058,21 @@
   </si>
   <si>
     <t>enum&lt;DuCurioExcitationPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioEncouragements</t>
+  </si>
+  <si>
+    <t>f4fe2c1acec5d8f0</t>
+  </si>
+  <si>
+    <t>crit_parameter</t>
+  </si>
+  <si>
+    <t>follow_up_crit_damage</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioEncouragementPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -13560,6 +13576,312 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="32.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: OriginalElationFollowUpDamage" promptTitle="DuCurioEncouragementPolicy enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
+      <formula1>"OriginalElationFollowUpDamage"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(universe): execute weighted curio dignity and passion policy
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -53,13 +53,14 @@
     <sheet name="BattleTeamResources" sheetId="44" r:id="rId44"/>
     <sheet name="WeightedCurioExcitations" sheetId="45" r:id="rId45"/>
     <sheet name="WeightedCurioEncouragements" sheetId="46" r:id="rId46"/>
+    <sheet name="WeightedCurioTransfers" sheetId="47" r:id="rId47"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3558" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3668" uniqueCount="347">
   <si>
     <t>@table</t>
   </si>
@@ -1073,6 +1074,33 @@
   </si>
   <si>
     <t>enum&lt;DuCurioEncouragementPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioTransfers</t>
+  </si>
+  <si>
+    <t>64ac6b5d093629d3</t>
+  </si>
+  <si>
+    <t>transfer_parameter</t>
+  </si>
+  <si>
+    <t>transfer_fraction</t>
+  </si>
+  <si>
+    <t>threshold_parameter</t>
+  </si>
+  <si>
+    <t>threshold_fraction</t>
+  </si>
+  <si>
+    <t>decay_parameter</t>
+  </si>
+  <si>
+    <t>decay_fraction</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioTransferPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -13882,6 +13910,425 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="14.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="13.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="27.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="21.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="6">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="M8:M1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: OtherShieldAppliedOwnerTurnExcessDecay" promptTitle="DuCurioTransferPolicy enum" prompt="Select a value from the dropdown." sqref="O8:O1007">
+      <formula1>"OtherShieldAppliedOwnerTurnExcessDecay"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(data): lower weighted curio overflow source operands
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -54,13 +54,14 @@
     <sheet name="WeightedCurioExcitations" sheetId="45" r:id="rId45"/>
     <sheet name="WeightedCurioEncouragements" sheetId="46" r:id="rId46"/>
     <sheet name="WeightedCurioTransfers" sheetId="47" r:id="rId47"/>
+    <sheet name="WeightedCurioOverflows" sheetId="48" r:id="rId48"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3668" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3768" uniqueCount="359">
   <si>
     <t>@table</t>
   </si>
@@ -1101,6 +1102,42 @@
   </si>
   <si>
     <t>enum&lt;DuCurioTransferPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioOverflows</t>
+  </si>
+  <si>
+    <t>7a414d6be44b58ed</t>
+  </si>
+  <si>
+    <t>base_parameter</t>
+  </si>
+  <si>
+    <t>base_multiplier</t>
+  </si>
+  <si>
+    <t>overflow_parameter</t>
+  </si>
+  <si>
+    <t>overflow_multiplier</t>
+  </si>
+  <si>
+    <t>attack_parameter</t>
+  </si>
+  <si>
+    <t>attack_increase</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>source_semantics</t>
+  </si>
+  <si>
+    <t>unresolved_runtime</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioOverflowStatus&gt;</t>
   </si>
 </sst>
 </file>
@@ -14329,6 +14366,388 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="19.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="18.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: PendingNativeDeathCallbackAndBaseDamage" promptTitle="DuCurioOverflowStatus enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"PendingNativeDeathCallbackAndBaseDamage"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>

</xml_diff>

<commit_message>
feat(data): author walkie-talkie base damage policy
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -55,13 +55,14 @@
     <sheet name="WeightedCurioEncouragements" sheetId="46" r:id="rId46"/>
     <sheet name="WeightedCurioTransfers" sheetId="47" r:id="rId47"/>
     <sheet name="WeightedCurioOverflows" sheetId="48" r:id="rId48"/>
+    <sheet name="WeightedCurioOverflowLevels" sheetId="49" r:id="rId49"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3768" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3843" uniqueCount="371">
   <si>
     <t>@table</t>
   </si>
@@ -1107,7 +1108,7 @@
     <t>DuWeightedCurioOverflows</t>
   </si>
   <si>
-    <t>7a414d6be44b58ed</t>
+    <t>ad5f29c71db84e40</t>
   </si>
   <si>
     <t>base_parameter</t>
@@ -1137,7 +1138,43 @@
     <t>unresolved_runtime</t>
   </si>
   <si>
+    <t>base_fixed_damage</t>
+  </si>
+  <si>
+    <t>base_hard_level_group</t>
+  </si>
+  <si>
+    <t>base_policy</t>
+  </si>
+  <si>
+    <t>base_policy_note</t>
+  </si>
+  <si>
+    <t>base_replacement_condition</t>
+  </si>
+  <si>
     <t>enum&lt;DuCurioOverflowStatus&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioOverflowBasePolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioOverflowLevels</t>
+  </si>
+  <si>
+    <t>a9398377cd8e966e</t>
+  </si>
+  <si>
+    <t>hard_level_group</t>
+  </si>
+  <si>
+    <t>unit_level</t>
+  </si>
+  <si>
+    <t>hp_ratio</t>
+  </si>
+  <si>
+    <t>range=1..95</t>
   </si>
 </sst>
 </file>
@@ -1789,8 +1826,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ObservedCommunity" promptTitle="DuDecisionEvidence enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"ExactStructured,ObservedCommunity"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ObservedCommunity, ProjectPolicy" promptTitle="DuDecisionEvidence enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"ExactStructured,ObservedCommunity,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14368,7 +14405,7 @@
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -14388,9 +14425,14 @@
     <col min="16" max="16" width="16.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="18.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="31.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="17.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="21.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="31.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" style="5" customWidth="1"/>
+    <col min="23" max="23" width="26.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14422,7 +14464,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="24" customHeight="1">
+    <row r="2" spans="1:23" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -14477,8 +14519,23 @@
       <c r="R2" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:18">
+      <c r="S2" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
@@ -14533,8 +14590,23 @@
       <c r="R3" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:18">
+      <c r="S3" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
       <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
@@ -14572,7 +14644,7 @@
         <v>23</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>23</v>
@@ -14589,8 +14661,23 @@
       <c r="R4" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:18">
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -14645,8 +14732,23 @@
       <c r="R5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:18">
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
       <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
@@ -14699,8 +14801,21 @@
       <c r="R6" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
@@ -14721,9 +14836,14 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
@@ -14742,6 +14862,219 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: PendingNativeDeathCallbackAndBaseDamage" promptTitle="DuCurioOverflowStatus enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"PendingNativeDeathCallbackAndBaseDamage"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 1." promptTitle="Integer range" prompt="Enter an integer from 1 to 1." sqref="T8:T1007">
+      <formula1>1</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: EnemyGroupOneHpRatioProtocolHpMultiplierFloor" promptTitle="DuCurioOverflowBasePolicy enum" prompt="Select a value from the dropdown." sqref="U8:U1007">
+      <formula1>"EnemyGroupOneHpRatioProtocolHpMultiplierFloor"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="12.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 1." promptTitle="Integer range" prompt="Enter an integer from 1 to 1." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 95." promptTitle="Integer range" prompt="Enter an integer from 1 to 95." sqref="F8:F1007">
+      <formula1>1</formula1>
+      <formula2>95</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(universe): admit walkie-talkie equipment policies
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3843" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3848" uniqueCount="372">
   <si>
     <t>@table</t>
   </si>
@@ -1108,7 +1108,7 @@
     <t>DuWeightedCurioOverflows</t>
   </si>
   <si>
-    <t>ad5f29c71db84e40</t>
+    <t>3d10e08827b592a6</t>
   </si>
   <si>
     <t>base_parameter</t>
@@ -1135,7 +1135,7 @@
     <t>source_semantics</t>
   </si>
   <si>
-    <t>unresolved_runtime</t>
+    <t>runtime_policy_note</t>
   </si>
   <si>
     <t>base_fixed_damage</t>
@@ -1151,6 +1151,9 @@
   </si>
   <si>
     <t>base_replacement_condition</t>
+  </si>
+  <si>
+    <t>runtime_replacement_condition</t>
   </si>
   <si>
     <t>enum&lt;DuCurioOverflowStatus&gt;</t>
@@ -14405,7 +14408,7 @@
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -14423,16 +14426,17 @@
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="16.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="19.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="31.7109375" style="5" customWidth="1"/>
     <col min="19" max="19" width="17.7109375" style="5" customWidth="1"/>
     <col min="20" max="20" width="21.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="31.7109375" style="5" customWidth="1"/>
     <col min="22" max="22" width="16.7109375" style="5" customWidth="1"/>
     <col min="23" max="23" width="26.7109375" style="5" customWidth="1"/>
+    <col min="24" max="24" width="29.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14464,7 +14468,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="24" customHeight="1">
+    <row r="2" spans="1:24" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -14534,8 +14538,11 @@
       <c r="W2" s="3" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="3" spans="1:23">
+      <c r="X2" s="3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
@@ -14605,8 +14612,11 @@
       <c r="W3" s="5" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="4" spans="1:23">
+      <c r="X3" s="5" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24">
       <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
@@ -14644,7 +14654,7 @@
         <v>23</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>23</v>
@@ -14668,7 +14678,7 @@
         <v>22</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="V4" s="5" t="s">
         <v>23</v>
@@ -14676,8 +14686,11 @@
       <c r="W4" s="5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:23">
+      <c r="X4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -14747,8 +14760,11 @@
       <c r="W5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:23">
+      <c r="X5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24">
       <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
@@ -14814,8 +14830,11 @@
       <c r="W6" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" ht="42" customHeight="1">
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
@@ -14841,6 +14860,7 @@
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="7">
@@ -14860,8 +14880,8 @@
       <formula1>1</formula1>
       <formula2>64</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: PendingNativeDeathCallbackAndBaseDamage" promptTitle="DuCurioOverflowStatus enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
-      <formula1>"PendingNativeDeathCallbackAndBaseDamage"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: NativeProjectPolicyHitEnded" promptTitle="DuCurioOverflowStatus enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"NativeProjectPolicyHitEnded"</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 1." promptTitle="Integer range" prompt="Enter an integer from 1 to 1." sqref="T8:T1007">
       <formula1>1</formula1>
@@ -14893,7 +14913,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14917,7 +14937,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -14934,13 +14954,13 @@
         <v>248</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>36</v>
@@ -14960,13 +14980,13 @@
         <v>248</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>36</v>
@@ -15041,7 +15061,7 @@
         <v>110</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat(divergent-universe): bind authored footstep equipment policies
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -56,13 +56,14 @@
     <sheet name="WeightedCurioTransfers" sheetId="47" r:id="rId47"/>
     <sheet name="WeightedCurioOverflows" sheetId="48" r:id="rId48"/>
     <sheet name="WeightedCurioOverflowLevels" sheetId="49" r:id="rId49"/>
+    <sheet name="WeightedCurioFootsteps" sheetId="50" r:id="rId50"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3848" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3958" uniqueCount="384">
   <si>
     <t>@table</t>
   </si>
@@ -1178,6 +1179,42 @@
   </si>
   <si>
     <t>range=1..95</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioFootsteps</t>
+  </si>
+  <si>
+    <t>8da07b1886f5e3f3</t>
+  </si>
+  <si>
+    <t>loss_parameter</t>
+  </si>
+  <si>
+    <t>loss_fraction</t>
+  </si>
+  <si>
+    <t>damage_per_stack</t>
+  </si>
+  <si>
+    <t>cap_parameter</t>
+  </si>
+  <si>
+    <t>maximum_stacks</t>
+  </si>
+  <si>
+    <t>hp_policy_note</t>
+  </si>
+  <si>
+    <t>hp_replacement_condition</t>
+  </si>
+  <si>
+    <t>skill_policy_note</t>
+  </si>
+  <si>
+    <t>skill_replacement_condition</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCurioFootstepPolicy&gt;</t>
   </si>
 </sst>
 </file>
@@ -15334,6 +15371,425 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" style="5" customWidth="1"/>
+    <col min="9" max="10" width="16.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="24.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="17.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="27.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="6">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="G8:G1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="I8:I1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 64." promptTitle="Integer range" prompt="Enter an integer from 1 to 64." sqref="K8:K1007">
+      <formula1>1</formula1>
+      <formula2>64</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 65535." promptTitle="Integer range" prompt="Enter an integer from 1 to 65535." sqref="L8:L1007">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: EffectiveHpLossAfterSkillOriginalDamage" promptTitle="DuCurioFootstepPolicy enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"EffectiveHpLossAfterSkillOriginalDamage"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q7"/>

</xml_diff>

<commit_message>
feat(data): author divergent universe deflagration operands
Bind six released Most Raucous operands and 95 exact HPRatios to pinned sources. Keep independently hashed base and execution policies explicit and native battle admission pending.

Regenerate the Sora schema, workbook and bundle together, validate typed loading and malformed inputs, and refresh configuration-bound public route vectors without weakening behavior assertions.
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -57,13 +57,15 @@
     <sheet name="WeightedCurioOverflows" sheetId="48" r:id="rId48"/>
     <sheet name="WeightedCurioOverflowLevels" sheetId="49" r:id="rId49"/>
     <sheet name="WeightedCurioFootsteps" sheetId="50" r:id="rId50"/>
+    <sheet name="WeightedCurioDeflagrations" sheetId="51" r:id="rId51"/>
+    <sheet name="WeightedCurioDeflagrationLevels" sheetId="52" r:id="rId52"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3958" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4132" uniqueCount="397">
   <si>
     <t>@table</t>
   </si>
@@ -1215,6 +1217,45 @@
   </si>
   <si>
     <t>enum&lt;DuCurioFootstepPolicy&gt;</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioDeflagrations</t>
+  </si>
+  <si>
+    <t>172135f6409c36b8</t>
+  </si>
+  <si>
+    <t>elements</t>
+  </si>
+  <si>
+    <t>burn_fractions</t>
+  </si>
+  <si>
+    <t>damage_multiplier</t>
+  </si>
+  <si>
+    <t>enum&lt;DuDeflagrationStatus&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuDeflagrationPolicy&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuDeflagrationBasePolicy&gt;</t>
+  </si>
+  <si>
+    <t>range=5..5</t>
+  </si>
+  <si>
+    <t>range=6..6</t>
+  </si>
+  <si>
+    <t>range=2..2</t>
+  </si>
+  <si>
+    <t>DuWeightedCurioDeflagrationLevels</t>
+  </si>
+  <si>
+    <t>54d8a1dd8dde51ca</t>
   </si>
 </sst>
 </file>
@@ -15790,6 +15831,683 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:W7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="6" width="12.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" style="5" customWidth="1"/>
+    <col min="14" max="15" width="26.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="30.7109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="19.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="29.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="16.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="26.7109375" style="5" customWidth="1"/>
+    <col min="23" max="23" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="8">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 5 to 5." promptTitle="Integer range" prompt="Enter an integer from 5 to 5." sqref="H8:H1007">
+      <formula1>5</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 6 to 6." promptTitle="Integer range" prompt="Enter an integer from 6 to 6." sqref="J8:J1007">
+      <formula1>6</formula1>
+      <formula2>6</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 2 to 2." promptTitle="Integer range" prompt="Enter an integer from 2 to 2." sqref="K8:K1007">
+      <formula1>2</formula1>
+      <formula2>2</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 1." promptTitle="Integer range" prompt="Enter an integer from 1 to 1." sqref="M8:M1007">
+      <formula1>1</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AuthoredOperandsPendingNative" promptTitle="DuDeflagrationStatus enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+      <formula1>"AuthoredOperandsPendingNative"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: OriginalFireAfterActionNaturalTickBurns" promptTitle="DuDeflagrationPolicy enum" prompt="Select a value from the dropdown." sqref="O8:O1007">
+      <formula1>"OriginalFireAfterActionNaturalTickBurns"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: TargetGroupOneHpRatioProtocolHpFloor" promptTitle="DuDeflagrationBasePolicy enum" prompt="Select a value from the dropdown." sqref="P8:P1007">
+      <formula1>"TargetGroupOneHpRatioProtocolHpFloor"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="12.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 1." promptTitle="Integer range" prompt="Enter an integer from 1 to 1." sqref="E8:E1007">
+      <formula1>1</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 95." promptTitle="Integer range" prompt="Enter an integer from 1 to 95." sqref="F8:F1007">
+      <formula1>1</formula1>
+      <formula2>95</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q7"/>

</xml_diff>

<commit_message>
feat(universe): admit deflagration equipment policy
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions-generated/templates/DivergentUniverseDecisions.xlsx
@@ -16288,8 +16288,8 @@
       <formula1>1</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AuthoredOperandsPendingNative" promptTitle="DuDeflagrationStatus enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
-      <formula1>"AuthoredOperandsPendingNative"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: NativeProjectPolicy" promptTitle="DuDeflagrationStatus enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+      <formula1>"NativeProjectPolicy"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: OriginalFireAfterActionNaturalTickBurns" promptTitle="DuDeflagrationPolicy enum" prompt="Select a value from the dropdown." sqref="O8:O1007">
       <formula1>"OriginalFireAfterActionNaturalTickBurns"</formula1>

</xml_diff>